<commit_message>
Tambah kolom Desil dengan dropdown 1-10 di Profil Mitra & SPPG
Co-authored-by: sppgbattuwinangun-lang <283471007+sppgbattuwinangun-lang@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Profil Mitra  SPPG.xlsx
+++ b/Profil Mitra  SPPG.xlsx
@@ -218,6 +218,7 @@
     <col min="15" max="15" width="32.400000000000006" customWidth="1"/>
     <col min="16" max="16" width="8.100000000000001" customWidth="1"/>
     <col min="17" max="17" width="6" customWidth="1"/>
+    <col min="19" max="19" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -313,6 +314,11 @@
           <t xml:space="preserve">Aksi</t>
         </is>
       </c>
+      <c t="inlineStr" r="S2" s="2">
+        <is>
+          <t xml:space="preserve">Desil</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="B3" s="65">
@@ -3766,8 +3772,13 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pilih Desil" prompt="Pilih nilai desil 1 sampai 10" errorTitle="Nilai tidak valid" error="Nilai harus antara 1 sampai 10" sqref="S3:S100">
+      <formula1>"1,2,3,4,5,6,7,8,9,10"</formula1>
+    </dataValidation>
+  </dataValidations>
   <mergeCells count="1">
-    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="A1:S1"/>
   </mergeCells>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix: betulkan urutan elemen XML mergeCells sebelum dataValidations
</commit_message>
<xml_diff>
--- a/Profil Mitra  SPPG.xlsx
+++ b/Profil Mitra  SPPG.xlsx
@@ -3772,13 +3772,13 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:S1"/>
+  </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pilih Desil" prompt="Pilih nilai desil 1 sampai 10" errorTitle="Nilai tidak valid" error="Nilai harus antara 1 sampai 10" sqref="S3:S100">
       <formula1>"1,2,3,4,5,6,7,8,9,10"</formula1>
     </dataValidation>
   </dataValidations>
-  <mergeCells count="1">
-    <mergeCell ref="A1:S1"/>
-  </mergeCells>
 </worksheet>
 </file>
</xml_diff>